<commit_message>
Update project with game systems and UI components
</commit_message>
<xml_diff>
--- a/Assets/Documents/Implementation/game_stats_data.xlsx
+++ b/Assets/Documents/Implementation/game_stats_data.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\admin\Unity\FighterScrollGame\Assets\Documents\Implementation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC5C7F2B-8F51-407B-B1B0-B1C208A8E916}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5089093-AE52-4D1E-819C-ADF084E67EC4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -661,7 +661,7 @@
         <v>60</v>
       </c>
       <c r="D2">
-        <v>100</v>
+        <v>3</v>
       </c>
       <c r="E2" t="s">
         <v>7</v>
@@ -757,7 +757,7 @@
         <v>6</v>
       </c>
       <c r="D8">
-        <v>100</v>
+        <v>3</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
@@ -841,7 +841,7 @@
         <v>60</v>
       </c>
       <c r="D14">
-        <v>100</v>
+        <v>3</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.3">

</xml_diff>